<commit_message>
Sismo R2.9: celdas de captura en amarillo fuerte
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ns7QgNzAi3QoiHRE1oS8iD
</commit_message>
<xml_diff>
--- a/EspectrosSismo_Naves_ElSalvador_NTDS_ASCE_STAAD_R2.9.xlsx
+++ b/EspectrosSismo_Naves_ElSalvador_NTDS_ASCE_STAAD_R2.9.xlsx
@@ -3247,8 +3247,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
-        <bgColor rgb="FFFFF0E0"/>
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
     <fill>

</xml_diff>

<commit_message>
Excel R2.9: factor en la direccion del SPECTRUM con SCALE 981 fijo; notas cortas
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DXC88k2xtfXzDpyA8FhCSg
</commit_message>
<xml_diff>
--- a/EspectrosSismo_Naves_ElSalvador_NTDS_ASCE_STAAD_R2.9.xlsx
+++ b/EspectrosSismo_Naves_ElSalvador_NTDS_ASCE_STAAD_R2.9.xlsx
@@ -14070,7 +14070,7 @@
       </c>
       <c r="F76" s="52" t="inlineStr">
         <is>
-          <t>◀ ESTE ES EL FACTOR. Multiplica el SCALE que ya tienes en el .STD (981 en el R2.9): SCALE nuevo = 981 × factor (fila 78). No es meter otra vez 981 encima: el 981 sólo pasa de g a cm/s². X en los casos 4 y 6; Z en los casos 5 y 7. Sube en la misma proporción todo lo del sismo: fuerzas, momentos, reacciones y desplazamientos.</t>
+          <t>◀ Factor que va en la dirección del SPECTRUM.</t>
         </is>
       </c>
       <c r="G76" s="48" t="inlineStr">
@@ -14082,7 +14082,7 @@
     <row r="77" ht="66" customHeight="1">
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>SCALE que traes en el .STD</t>
+          <t>SCALE en STAAD</t>
         </is>
       </c>
       <c r="C77" s="16">
@@ -14098,28 +14098,28 @@
       </c>
       <c r="F77" s="44" t="inlineStr">
         <is>
-          <t>CAPTURA. El SCALE que hoy tienen los SPECTRUM de tu .STD. R2.9: 981, porque la lista que pegaste ya viene en g y dividida entre R (meseta 0.2057 g); el 981 sólo convierte g a cm/s². Si usas la lista ELÁSTICA de la hoja STAAD (meseta 1.44 g, como el R3.2), aquí va 140.095 = 980.665/7.</t>
+          <t>Fijo: g → cm/s².</t>
         </is>
       </c>
       <c r="G77" s="48" t="inlineStr">
         <is>
-          <t>Archivo .STD (R2.9: líneas 565, 585, 605 y 625)</t>
+          <t>Archivo .STD</t>
         </is>
       </c>
     </row>
     <row r="78" ht="30" customHeight="1">
       <c r="B78" s="8" t="inlineStr">
         <is>
-          <t>SCALE nuevo = SCALE × factor</t>
+          <t>Factor de dirección en SPECTRUM</t>
         </is>
       </c>
       <c r="C78" s="21">
-        <f>$C$77*$C$76</f>
-        <v>1590.3079405241106</v>
+        <f>$C$76</f>
+        <v>1.6211090117473095</v>
       </c>
       <c r="D78" s="21">
-        <f>$D$77*$D$76</f>
-        <v>1107.9087702910244</v>
+        <f>$D$76</f>
+        <v>1.129366738319087</v>
       </c>
       <c r="E78" s="6" t="inlineStr">
         <is>
@@ -14128,7 +14128,7 @@
       </c>
       <c r="F78" s="44" t="inlineStr">
         <is>
-          <t>CALCULADA = SCALE actual × factor. Es el número que escribes en SPECTRUM ... ACC SCALE: X en los casos 4 y 6; Z en los casos 5 y 7.</t>
+          <t>X: caso 4 (+), caso 6 (−). Z: caso 5 (+), caso 7 (−).</t>
         </is>
       </c>
       <c r="G78" s="48" t="inlineStr">
@@ -14158,7 +14158,7 @@
       </c>
       <c r="F79" s="44" t="inlineStr">
         <is>
-          <t>CALCULADA. Para la deriva se quita el 80% del Método A y vale el T del modelo (Método B).</t>
+          <t>CALCULADA.</t>
         </is>
       </c>
       <c r="G79" s="48" t="inlineStr">
@@ -14188,7 +14188,7 @@
       </c>
       <c r="F80" s="44" t="inlineStr">
         <is>
-          <t>CALCULADA. Deriva = δ del modelo sin escalar × C_d × este factor.</t>
+          <t>Deriva = δ × C_d × factor.</t>
         </is>
       </c>
       <c r="G80" s="48" t="inlineStr">
@@ -14212,7 +14212,7 @@
     <row r="83" ht="42" customHeight="1">
       <c r="B83" s="35" t="inlineStr">
         <is>
-          <t>Las dos hojas usan el mismo método (NTDS §5.4.1-3): V mínimo = el mayor de 90% del estático con el T del modelo y 80% del de Método A; factor = V mínimo / V modal. Los factores no salen iguales porque cambian W, T y el V modal. Los valores de él están en azul, copiados de su archivo.</t>
+          <t>Mismo método en las dos. Valores de él en azul.</t>
         </is>
       </c>
       <c r="C83" s="35"/>
@@ -14285,7 +14285,7 @@
       </c>
       <c r="F86" s="44" t="inlineStr">
         <is>
-          <t>Ya igualado: los dos usan el peso de STAAD (17.13 t). Esta diferencia ya no existe.</t>
+          <t>Ya igualado (peso de STAAD).</t>
         </is>
       </c>
       <c r="G86" s="48" t="inlineStr">
@@ -14314,7 +14314,7 @@
       </c>
       <c r="F87" s="44" t="inlineStr">
         <is>
-          <t>Él lo redondea a 2 decimales para buscar C_sm en su tabla. Viene de otra corrida del modelo.</t>
+          <t>Él redondea a 2 decimales.</t>
         </is>
       </c>
       <c r="G87" s="48" t="inlineStr">
@@ -14343,7 +14343,7 @@
       </c>
       <c r="F88" s="44" t="inlineStr">
         <is>
-          <t>Misma ecuación 4.2 de la NTDS; cambia sólo porque cambia T.</t>
+          <t>Misma ec. 4.2.</t>
         </is>
       </c>
       <c r="G88" s="48" t="inlineStr">
@@ -14373,7 +14373,7 @@
       </c>
       <c r="F89" s="44" t="inlineStr">
         <is>
-          <t>Igual en las dos: 0.8 × 0.2057 (él usa T = T_o = 0.6 s; tú 0.479 s, que la norma sube a T_o).</t>
+          <t>Igual en las dos.</t>
         </is>
       </c>
       <c r="G89" s="48" t="inlineStr">
@@ -14403,7 +14403,7 @@
       </c>
       <c r="F90" s="44" t="inlineStr">
         <is>
-          <t>El mayor de 90% del C_s con T y 80% del de Método A.</t>
+          <t>Mayor de 90% C_s(T) y 80% Método A.</t>
         </is>
       </c>
       <c r="G90" s="48" t="inlineStr">
@@ -14433,7 +14433,7 @@
       </c>
       <c r="F91" s="44" t="inlineStr">
         <is>
-          <t>C_s mínimo × W: aquí entra la diferencia de W.</t>
+          <t>C_s mínimo × W.</t>
         </is>
       </c>
       <c r="G91" s="48" t="inlineStr">
@@ -14462,7 +14462,7 @@
       </c>
       <c r="F92" s="44" t="inlineStr">
         <is>
-          <t>Tú: el cortante que imprime STAAD en el .anl (CQC). Él: lo recalcula a mano con C_sm(T)·W·%masa de cada modo y SRSS, con T redondeado. Para el factor vale el de STAAD.</t>
+          <t>Tú: STAAD (.anl). Él: a mano. Vale el de STAAD.</t>
         </is>
       </c>
       <c r="G92" s="48" t="inlineStr">
@@ -14492,7 +14492,7 @@
       </c>
       <c r="F93" s="44" t="inlineStr">
         <is>
-          <t>El tuyo es el verde de la fila 76. El de él sale menor porque su V modal es mayor y su W menor.</t>
+          <t>Fila 76.</t>
         </is>
       </c>
       <c r="G93" s="48" t="inlineStr">
@@ -14533,7 +14533,7 @@
       </c>
       <c r="F95" s="44" t="inlineStr">
         <is>
-          <t>Ya igualado: los dos usan el peso de STAAD (17.13 t). Esta diferencia ya no existe.</t>
+          <t>Ya igualado (peso de STAAD).</t>
         </is>
       </c>
       <c r="G95" s="48" t="inlineStr">
@@ -14562,7 +14562,7 @@
       </c>
       <c r="F96" s="44" t="inlineStr">
         <is>
-          <t>Él lo redondea a 2 decimales para buscar C_sm en su tabla. Viene de otra corrida del modelo.</t>
+          <t>Él redondea a 2 decimales.</t>
         </is>
       </c>
       <c r="G96" s="48" t="inlineStr">
@@ -14591,7 +14591,7 @@
       </c>
       <c r="F97" s="44" t="inlineStr">
         <is>
-          <t>Misma ecuación 4.2 de la NTDS; cambia sólo porque cambia T.</t>
+          <t>Misma ec. 4.2.</t>
         </is>
       </c>
       <c r="G97" s="48" t="inlineStr">
@@ -14621,7 +14621,7 @@
       </c>
       <c r="F98" s="44" t="inlineStr">
         <is>
-          <t>Igual en las dos: 0.8 × 0.2057 (él usa T = T_o = 0.6 s; tú 0.479 s, que la norma sube a T_o).</t>
+          <t>Igual en las dos.</t>
         </is>
       </c>
       <c r="G98" s="48" t="inlineStr">
@@ -14651,7 +14651,7 @@
       </c>
       <c r="F99" s="44" t="inlineStr">
         <is>
-          <t>El mayor de 90% del C_s con T y 80% del de Método A.</t>
+          <t>Mayor de 90% C_s(T) y 80% Método A.</t>
         </is>
       </c>
       <c r="G99" s="48" t="inlineStr">
@@ -14681,7 +14681,7 @@
       </c>
       <c r="F100" s="44" t="inlineStr">
         <is>
-          <t>C_s mínimo × W: aquí entra la diferencia de W.</t>
+          <t>C_s mínimo × W.</t>
         </is>
       </c>
       <c r="G100" s="48" t="inlineStr">
@@ -14710,7 +14710,7 @@
       </c>
       <c r="F101" s="44" t="inlineStr">
         <is>
-          <t>Tú: el cortante que imprime STAAD en el .anl (CQC). Él: lo recalcula a mano con C_sm(T)·W·%masa de cada modo y SRSS, con T redondeado. Para el factor vale el de STAAD.</t>
+          <t>Tú: STAAD (.anl). Él: a mano. Vale el de STAAD.</t>
         </is>
       </c>
       <c r="G101" s="48" t="inlineStr">
@@ -14740,7 +14740,7 @@
       </c>
       <c r="F102" s="44" t="inlineStr">
         <is>
-          <t>El tuyo es el verde de la fila 76. El de él sale menor porque su V modal es mayor y su W menor.</t>
+          <t>Fila 76.</t>
         </is>
       </c>
       <c r="G102" s="48" t="inlineStr">
@@ -14752,7 +14752,7 @@
     <row r="103" ht="30" customHeight="1">
       <c r="B103" s="45" t="inlineStr">
         <is>
-          <t>Cómo meter el factor en STAAD (las dos formas dan lo mismo)</t>
+          <t>Cómo queda en STAAD (SCALE 981)</t>
         </is>
       </c>
       <c r="C103" s="45" t="inlineStr">
@@ -14784,16 +14784,16 @@
     <row r="104" ht="42" customHeight="1">
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>R2.9 — lista de DISEÑO ÷R (meseta 0.2057 g), SCALE 981: SCALE nuevo</t>
+          <t>Factor de dirección, casos 4 y 5</t>
         </is>
       </c>
       <c r="C104" s="13">
-        <f>$C$78</f>
-        <v>1590.3079405241106</v>
+        <f>$C$76</f>
+        <v>1.6211090117473095</v>
       </c>
       <c r="D104" s="13">
-        <f>$D$78</f>
-        <v>1107.9087702910244</v>
+        <f>$D$76</f>
+        <v>1.129366738319087</v>
       </c>
       <c r="E104" s="6" t="inlineStr">
         <is>
@@ -14802,28 +14802,28 @@
       </c>
       <c r="F104" s="44" t="inlineStr">
         <is>
-          <t>981 × factor. Es lo que va en tu .STD R2.9.</t>
+          <t>Positivo.</t>
         </is>
       </c>
       <c r="G104" s="48" t="inlineStr">
         <is>
-          <t>Fila 78</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="105" ht="42" customHeight="1">
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>Lista ELÁSTICA de la hoja STAAD (meseta 1.44 g), SCALE 140.095: SCALE nuevo</t>
+          <t>Factor de dirección, casos 6 y 7</t>
         </is>
       </c>
       <c r="C105" s="13">
-        <f>STAAD!$C$18*$C$76</f>
-        <v>227.10926700073932</v>
+        <f>-$C$76</f>
+        <v>-1.6211090117473095</v>
       </c>
       <c r="D105" s="13">
-        <f>STAAD!$D$18*$D$76</f>
-        <v>158.2186332048125</v>
+        <f>-$D$76</f>
+        <v>-1.129366738319087</v>
       </c>
       <c r="E105" s="6" t="inlineStr">
         <is>
@@ -14832,12 +14832,12 @@
       </c>
       <c r="F105" s="44" t="inlineStr">
         <is>
-          <t>140.095 × factor. Sólo si pegas la lista elástica (como el R3.2). NO lo mezcles con la lista ÷R del R2.9: saldría 7 veces más chico.</t>
+          <t>Negativo.</t>
         </is>
       </c>
       <c r="G105" s="48" t="inlineStr">
         <is>
-          <t>Hoja STAAD, C18</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -14862,7 +14862,7 @@
       </c>
       <c r="F106" s="44" t="inlineStr">
         <is>
-          <t>= 0.2057 g × factor. Las dos formas de arriba dan esta misma meseta.</t>
+          <t>0.2057 g × factor.</t>
         </is>
       </c>
       <c r="G106" s="48" t="inlineStr">

</xml_diff>

<commit_message>
Excel R2.9: notas cortas con origen (captura STAAD / calculada / fija) y referencia de norma
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DXC88k2xtfXzDpyA8FhCSg
</commit_message>
<xml_diff>
--- a/EspectrosSismo_Naves_ElSalvador_NTDS_ASCE_STAAD_R2.9.xlsx
+++ b/EspectrosSismo_Naves_ElSalvador_NTDS_ASCE_STAAD_R2.9.xlsx
@@ -12404,8 +12404,10 @@
       <c r="D58" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="E58" s="3" t="s">
-        <v>163</v>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>CAPTURA de STAAD: periodo del modo con mayor masa en X (.anl). Con 0 se usa el aproximado.</t>
+        </is>
       </c>
       <c r="F58" s="4" t="s">
         <v>164</v>
@@ -12421,8 +12423,10 @@
       <c r="D59" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="E59" s="3" t="s">
-        <v>166</v>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>CAPTURA de STAAD: periodo del modo con mayor masa en Z (.anl). Con 0 se usa el aproximado.</t>
+        </is>
       </c>
       <c r="F59" s="4" t="s">
         <v>164</v>
@@ -12440,7 +12444,7 @@
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>CAPTURA. 17.13 t = peso sísmico que reporta STAAD (el mismo que usa ANALISIS_CARGAS_NAVE, 17,129 kg), para que el V mínimo y el V modal salgan de la misma masa. Antes: 17.49 t por áreas tributarias (acero 11.82 + CM techo 3.12 + CM muros 2.15 + cortina 0.40).</t>
+          <t>CAPTURA de STAAD: DYNAMIC WEIGHT X Y Z = 17,128.09 kg (.anl).</t>
         </is>
       </c>
       <c r="F60" s="4" t="s">
@@ -12459,7 +12463,7 @@
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>CAPTURA. Igual que la NTDS: 17.13 t (fuera del AMSS sólo es referencia).</t>
+          <t>CAPTURA de STAAD: igual que la NTDS.</t>
         </is>
       </c>
       <c r="F61" s="4" t="s">
@@ -13980,12 +13984,12 @@
       </c>
       <c r="F73" s="44" t="inlineStr">
         <is>
-          <t>CAPTURA. Del .anl: TOTAL SRSS SHEAR del caso 4 (X) y del caso 5 (Z), en kg ÷ 1000.</t>
+          <t>CAPTURA de STAAD: cortante basal SRSS del caso 4 (X) y 5 (Z) en el .anl, kg ÷ 1000.</t>
         </is>
       </c>
       <c r="G73" s="48" t="inlineStr">
         <is>
-          <t>Salida de STAAD</t>
+          <t>Salida de STAAD (.anl)</t>
         </is>
       </c>
     </row>
@@ -14070,7 +14074,7 @@
       </c>
       <c r="F76" s="52" t="inlineStr">
         <is>
-          <t>◀ Factor que va en la dirección del SPECTRUM.</t>
+          <t>◀ CALCULADA = V mín / V dinámico. Va en la dirección del SPECTRUM.</t>
         </is>
       </c>
       <c r="G76" s="48" t="inlineStr">
@@ -14098,12 +14102,12 @@
       </c>
       <c r="F77" s="44" t="inlineStr">
         <is>
-          <t>Fijo: g → cm/s².</t>
+          <t>FIJO. Convierte g a cm/s² (modelo en kg-cm).</t>
         </is>
       </c>
       <c r="G77" s="48" t="inlineStr">
         <is>
-          <t>Archivo .STD</t>
+          <t>Archivo .STD R2.9 · casos 4 a 7</t>
         </is>
       </c>
     </row>
@@ -14128,12 +14132,12 @@
       </c>
       <c r="F78" s="44" t="inlineStr">
         <is>
-          <t>X: caso 4 (+), caso 6 (−). Z: caso 5 (+), caso 7 (−).</t>
+          <t>= fila 76. X: caso 4 (+), 6 (−). Z: caso 5 (+), 7 (−).</t>
         </is>
       </c>
       <c r="G78" s="48" t="inlineStr">
         <is>
-          <t>Archivo .STD</t>
+          <t>Manual técnico de STAAD.Pro · comando SPECTRUM</t>
         </is>
       </c>
     </row>
@@ -14158,7 +14162,7 @@
       </c>
       <c r="F79" s="44" t="inlineStr">
         <is>
-          <t>CALCULADA.</t>
+          <t>CALCULADA = 90% de C_s(T) × W, sin el 80% del Método A.</t>
         </is>
       </c>
       <c r="G79" s="48" t="inlineStr">
@@ -14188,12 +14192,12 @@
       </c>
       <c r="F80" s="44" t="inlineStr">
         <is>
-          <t>Deriva = δ × C_d × factor.</t>
+          <t>CALCULADA. Deriva = δ × C_d × factor.</t>
         </is>
       </c>
       <c r="G80" s="48" t="inlineStr">
         <is>
-          <t>NTDS-1994 · ec. 4.11 y §4.6.2, pág. 9</t>
+          <t>NTDS-1994 · ec. 4.11 y §4.6.2, pág. 9 · Tabla 8, pág. 24</t>
         </is>
       </c>
     </row>
@@ -14244,12 +14248,12 @@
       </c>
       <c r="F84" s="45" t="inlineStr">
         <is>
-          <t>Por qué difiere</t>
+          <t>De dónde sale</t>
         </is>
       </c>
       <c r="G84" s="45" t="inlineStr">
         <is>
-          <t>De dónde sale el valor de él</t>
+          <t>Referencia</t>
         </is>
       </c>
     </row>
@@ -14285,12 +14289,12 @@
       </c>
       <c r="F86" s="44" t="inlineStr">
         <is>
-          <t>Ya igualado (peso de STAAD).</t>
+          <t>Tú: CAPTURA de STAAD, DYNAMIC WEIGHT (.anl). Él: E165.</t>
         </is>
       </c>
       <c r="G86" s="48" t="inlineStr">
         <is>
-          <t>ANALISIS_CARGAS_NAVE.xlsx · CARGAS Y SISMO F1 · K197 / E165</t>
+          <t>NTDS-1994 · §4.1.3, pág. 7</t>
         </is>
       </c>
     </row>
@@ -14314,12 +14318,12 @@
       </c>
       <c r="F87" s="44" t="inlineStr">
         <is>
-          <t>Él redondea a 2 decimales.</t>
+          <t>Tú: CAPTURA de STAAD, periodo del modo en X (.anl). Él: D177, redondeado.</t>
         </is>
       </c>
       <c r="G87" s="48" t="inlineStr">
         <is>
-          <t>ANALISIS_CARGAS_NAVE.xlsx · CARGAS Y SISMO F1 · D177 (0.807 → 0.81)</t>
+          <t>NTDS-1994 · §4.2.2 (2), págs. 7 y 8</t>
         </is>
       </c>
     </row>
@@ -14343,12 +14347,12 @@
       </c>
       <c r="F88" s="44" t="inlineStr">
         <is>
-          <t>Misma ec. 4.2.</t>
+          <t>CALCULADA con el T de arriba. Él: J177.</t>
         </is>
       </c>
       <c r="G88" s="48" t="inlineStr">
         <is>
-          <t>ANALISIS_CARGAS_NAVE.xlsx · CARGAS Y SISMO F1 · J177</t>
+          <t>NTDS-1994 · ec. 4.2, pág. 7</t>
         </is>
       </c>
     </row>
@@ -14373,12 +14377,12 @@
       </c>
       <c r="F89" s="44" t="inlineStr">
         <is>
-          <t>Igual en las dos.</t>
+          <t>CALCULADA = 0.8 × A·I·C_o / R. Él: F141.</t>
         </is>
       </c>
       <c r="G89" s="48" t="inlineStr">
         <is>
-          <t>ANALISIS_CARGAS_NAVE.xlsx · CARGAS Y SISMO F1 · F141</t>
+          <t>NTDS-1994 · ec. 4.3, pág. 7 · §5.4.1 (3), pág. 12</t>
         </is>
       </c>
     </row>
@@ -14403,12 +14407,12 @@
       </c>
       <c r="F90" s="44" t="inlineStr">
         <is>
-          <t>Mayor de 90% C_s(T) y 80% Método A.</t>
+          <t>CALCULADA: mayor de 90% C_s(T) y 80% Método A. Él: K207 ÷ W.</t>
         </is>
       </c>
       <c r="G90" s="48" t="inlineStr">
         <is>
-          <t>ANALISIS_CARGAS_NAVE.xlsx · CARGAS Y SISMO F1 · K207 ÷ W</t>
+          <t>NTDS-1994 · §5.4.1 (3), pág. 12</t>
         </is>
       </c>
     </row>
@@ -14433,12 +14437,12 @@
       </c>
       <c r="F91" s="44" t="inlineStr">
         <is>
-          <t>C_s mínimo × W.</t>
+          <t>CALCULADA = C_s mín × W. Él: K211.</t>
         </is>
       </c>
       <c r="G91" s="48" t="inlineStr">
         <is>
-          <t>ANALISIS_CARGAS_NAVE.xlsx · CARGAS Y SISMO F1 · K211</t>
+          <t>NTDS-1994 · ec. 4.1, pág. 7 · §5.4.1 (3), pág. 12</t>
         </is>
       </c>
     </row>
@@ -14462,12 +14466,12 @@
       </c>
       <c r="F92" s="44" t="inlineStr">
         <is>
-          <t>Tú: STAAD (.anl). Él: a mano. Vale el de STAAD.</t>
+          <t>Tú: CAPTURA de STAAD, cortante SRSS del caso 4 (.anl). Él: K212, a mano.</t>
         </is>
       </c>
       <c r="G92" s="48" t="inlineStr">
         <is>
-          <t>ANALISIS_CARGAS_NAVE.xlsx · CARGAS Y SISMO F1 · K212</t>
+          <t>Salida de STAAD (.anl) · NTDS-1994 · §5.4.1 (3), pág. 12</t>
         </is>
       </c>
     </row>
@@ -14492,12 +14496,12 @@
       </c>
       <c r="F93" s="44" t="inlineStr">
         <is>
-          <t>Fila 76.</t>
+          <t>CALCULADA = V mín / V modal. Tú: fila 76. Él: K214.</t>
         </is>
       </c>
       <c r="G93" s="48" t="inlineStr">
         <is>
-          <t>ANALISIS_CARGAS_NAVE.xlsx · CARGAS Y SISMO F1 · K214</t>
+          <t>NTDS-1994 · §5.4.1 (3), pág. 12</t>
         </is>
       </c>
     </row>
@@ -14533,12 +14537,12 @@
       </c>
       <c r="F95" s="44" t="inlineStr">
         <is>
-          <t>Ya igualado (peso de STAAD).</t>
+          <t>Tú: CAPTURA de STAAD, DYNAMIC WEIGHT (.anl). Él: E165.</t>
         </is>
       </c>
       <c r="G95" s="48" t="inlineStr">
         <is>
-          <t>ANALISIS_CARGAS_NAVE.xlsx · CARGAS Y SISMO F1 · K197 / E165</t>
+          <t>NTDS-1994 · §4.1.3, pág. 7</t>
         </is>
       </c>
     </row>
@@ -14562,12 +14566,12 @@
       </c>
       <c r="F96" s="44" t="inlineStr">
         <is>
-          <t>Él redondea a 2 decimales.</t>
+          <t>Tú: CAPTURA de STAAD, periodo del modo en Z (.anl). Él: D178, redondeado.</t>
         </is>
       </c>
       <c r="G96" s="48" t="inlineStr">
         <is>
-          <t>ANALISIS_CARGAS_NAVE.xlsx · CARGAS Y SISMO F1 · D178 (0.628 → 0.63)</t>
+          <t>NTDS-1994 · §4.2.2 (2), págs. 7 y 8</t>
         </is>
       </c>
     </row>
@@ -14591,12 +14595,12 @@
       </c>
       <c r="F97" s="44" t="inlineStr">
         <is>
-          <t>Misma ec. 4.2.</t>
+          <t>CALCULADA con el T de arriba. Él: J178.</t>
         </is>
       </c>
       <c r="G97" s="48" t="inlineStr">
         <is>
-          <t>ANALISIS_CARGAS_NAVE.xlsx · CARGAS Y SISMO F1 · J178</t>
+          <t>NTDS-1994 · ec. 4.2, pág. 7</t>
         </is>
       </c>
     </row>
@@ -14621,12 +14625,12 @@
       </c>
       <c r="F98" s="44" t="inlineStr">
         <is>
-          <t>Igual en las dos.</t>
+          <t>CALCULADA = 0.8 × A·I·C_o / R. Él: F141.</t>
         </is>
       </c>
       <c r="G98" s="48" t="inlineStr">
         <is>
-          <t>ANALISIS_CARGAS_NAVE.xlsx · CARGAS Y SISMO F1 · F141</t>
+          <t>NTDS-1994 · ec. 4.3, pág. 7 · §5.4.1 (3), pág. 12</t>
         </is>
       </c>
     </row>
@@ -14651,12 +14655,12 @@
       </c>
       <c r="F99" s="44" t="inlineStr">
         <is>
-          <t>Mayor de 90% C_s(T) y 80% Método A.</t>
+          <t>CALCULADA: mayor de 90% C_s(T) y 80% Método A. Él: L207 ÷ W.</t>
         </is>
       </c>
       <c r="G99" s="48" t="inlineStr">
         <is>
-          <t>ANALISIS_CARGAS_NAVE.xlsx · CARGAS Y SISMO F1 · K207 ÷ W</t>
+          <t>NTDS-1994 · §5.4.1 (3), pág. 12</t>
         </is>
       </c>
     </row>
@@ -14681,12 +14685,12 @@
       </c>
       <c r="F100" s="44" t="inlineStr">
         <is>
-          <t>C_s mínimo × W.</t>
+          <t>CALCULADA = C_s mín × W. Él: L211.</t>
         </is>
       </c>
       <c r="G100" s="48" t="inlineStr">
         <is>
-          <t>ANALISIS_CARGAS_NAVE.xlsx · CARGAS Y SISMO F1 · L211</t>
+          <t>NTDS-1994 · ec. 4.1, pág. 7 · §5.4.1 (3), pág. 12</t>
         </is>
       </c>
     </row>
@@ -14710,12 +14714,12 @@
       </c>
       <c r="F101" s="44" t="inlineStr">
         <is>
-          <t>Tú: STAAD (.anl). Él: a mano. Vale el de STAAD.</t>
+          <t>Tú: CAPTURA de STAAD, cortante SRSS del caso 5 (.anl). Él: L212, a mano.</t>
         </is>
       </c>
       <c r="G101" s="48" t="inlineStr">
         <is>
-          <t>ANALISIS_CARGAS_NAVE.xlsx · CARGAS Y SISMO F1 · L212</t>
+          <t>Salida de STAAD (.anl) · NTDS-1994 · §5.4.1 (3), pág. 12</t>
         </is>
       </c>
     </row>
@@ -14740,12 +14744,12 @@
       </c>
       <c r="F102" s="44" t="inlineStr">
         <is>
-          <t>Fila 76.</t>
+          <t>CALCULADA = V mín / V modal. Tú: fila 76. Él: L214.</t>
         </is>
       </c>
       <c r="G102" s="48" t="inlineStr">
         <is>
-          <t>ANALISIS_CARGAS_NAVE.xlsx · CARGAS Y SISMO F1 · L214</t>
+          <t>NTDS-1994 · §5.4.1 (3), pág. 12</t>
         </is>
       </c>
     </row>
@@ -14772,7 +14776,7 @@
       </c>
       <c r="F103" s="45" t="inlineStr">
         <is>
-          <t>Cómo se calcula</t>
+          <t>De dónde sale</t>
         </is>
       </c>
       <c r="G103" s="45" t="inlineStr">
@@ -14802,12 +14806,12 @@
       </c>
       <c r="F104" s="44" t="inlineStr">
         <is>
-          <t>Positivo.</t>
+          <t>= fila 76, con signo +.</t>
         </is>
       </c>
       <c r="G104" s="48" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Manual técnico de STAAD.Pro · comando SPECTRUM</t>
         </is>
       </c>
     </row>
@@ -14832,12 +14836,12 @@
       </c>
       <c r="F105" s="44" t="inlineStr">
         <is>
-          <t>Negativo.</t>
+          <t>= fila 76, con signo −.</t>
         </is>
       </c>
       <c r="G105" s="48" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Manual técnico de STAAD.Pro · comando SPECTRUM</t>
         </is>
       </c>
     </row>
@@ -14862,12 +14866,12 @@
       </c>
       <c r="F106" s="44" t="inlineStr">
         <is>
-          <t>0.2057 g × factor.</t>
+          <t>CALCULADA = I·A·C_o / R × factor.</t>
         </is>
       </c>
       <c r="G106" s="48" t="inlineStr">
         <is>
-          <t>NTDS §5.2 y §5.4.1</t>
+          <t>NTDS-1994 · §5.2, pág. 11 · §5.4.1 (3), pág. 12</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
R3.0: espectro X 1.448 / Z 1.727 con W, T y V dinamico del .anl R3.0
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DXC88k2xtfXzDpyA8FhCSg
</commit_message>
<xml_diff>
--- a/EspectrosSismo_Naves_ElSalvador_NTDS_ASCE_STAAD_R2.9.xlsx
+++ b/EspectrosSismo_Naves_ElSalvador_NTDS_ASCE_STAAD_R2.9.xlsx
@@ -12399,7 +12399,7 @@
         <v>162</v>
       </c>
       <c r="C58" s="16">
-        <v>0.889</v>
+        <v>0.334</v>
       </c>
       <c r="D58" s="6" t="s">
         <v>79</v>
@@ -12418,7 +12418,7 @@
         <v>165</v>
       </c>
       <c r="C59" s="16">
-        <v>0.631</v>
+        <v>0.125</v>
       </c>
       <c r="D59" s="6" t="s">
         <v>79</v>
@@ -12437,14 +12437,14 @@
         <v>167</v>
       </c>
       <c r="C60" s="15">
-        <v>17.13</v>
+        <v>21.662</v>
       </c>
       <c r="D60" s="6" t="s">
         <v>168</v>
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>CAPTURA de STAAD: DYNAMIC WEIGHT X Y Z = 17,128.09 kg (.anl).</t>
+          <t>CAPTURA de STAAD: DYNAMIC WEIGHT X Y Z = 21,662.18 kg (.anl R3.0).</t>
         </is>
       </c>
       <c r="F60" s="4" t="s">
@@ -12456,7 +12456,7 @@
         <v>170</v>
       </c>
       <c r="C61" s="15">
-        <v>17.13</v>
+        <v>21.662</v>
       </c>
       <c r="D61" s="6" t="s">
         <v>168</v>
@@ -12908,11 +12908,11 @@
       </c>
       <c r="C19" s="13">
         <f>IF(DATOS!$C$58&gt;0,DATOS!$C$58,$C$18)</f>
-        <v>0.889</v>
+        <v>0.334</v>
       </c>
       <c r="D19" s="13">
         <f>IF(DATOS!$C$59&gt;0,DATOS!$C$59,$D$18)</f>
-        <v>0.631</v>
+        <v>0.125</v>
       </c>
       <c r="E19" s="6" t="s">
         <v>79</v>
@@ -12930,11 +12930,11 @@
       </c>
       <c r="C20" s="13">
         <f>MIN(MAX($C$19,DATOS!$C$23),6*DATOS!$C$23)</f>
-        <v>0.889</v>
+        <v>0.6</v>
       </c>
       <c r="D20" s="13">
         <f>MIN(MAX($D$19,DATOS!$C$23),6*DATOS!$C$23)</f>
-        <v>0.631</v>
+        <v>0.6</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>79</v>
@@ -12952,11 +12952,11 @@
       </c>
       <c r="C21" s="19">
         <f>DATOS!$C$20*DATOS!$C$25*DATOS!$C$22/$C$12*(DATOS!$C$23/$C$20)^(2/3)</f>
-        <v>0.15828172633756074</v>
+        <v>0.2057142857142857</v>
       </c>
       <c r="D21" s="19">
         <f>DATOS!$C$20*DATOS!$C$25*DATOS!$C$22/$D$12*(DATOS!$C$23/$D$20)^(2/3)</f>
-        <v>0.19892027280931626</v>
+        <v>0.2057142857142857</v>
       </c>
       <c r="E21" s="6" t="s">
         <v>43</v>
@@ -12996,11 +12996,11 @@
       </c>
       <c r="C23" s="20">
         <f>IF(DATOS!$C$58&gt;0,MAX($C$21,0.8*$C$22),$C$22)</f>
-        <v>0.1645714285714286</v>
+        <v>0.2057142857142857</v>
       </c>
       <c r="D23" s="20">
         <f>IF(DATOS!$C$59&gt;0,MAX($D$21,0.8*$D$22),$D$22)</f>
-        <v>0.19892027280931626</v>
+        <v>0.2057142857142857</v>
       </c>
       <c r="E23" s="6" t="s">
         <v>43</v>
@@ -13018,11 +13018,11 @@
       </c>
       <c r="C24" s="21">
         <f>$C$23*DATOS!$C$60</f>
-        <v>2.8191085714285715</v>
+        <v>4.456182857142857</v>
       </c>
       <c r="D24" s="21">
         <f>$D$23*DATOS!$C$60</f>
-        <v>3.407504273223587</v>
+        <v>4.456182857142857</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>168</v>
@@ -13040,7 +13040,7 @@
       </c>
       <c r="C25" s="13">
         <f>IF($C$19&lt;=0.7,0,MIN(0.07*$C$19,0.25))</f>
-        <v>0.06223000000000001</v>
+        <v>0.0</v>
       </c>
       <c r="D25" s="13">
         <f>IF($D$19&lt;=0.7,0,MIN(0.07*$D$19,0.25))</f>
@@ -13084,11 +13084,11 @@
       </c>
       <c r="C27" s="19">
         <f>IF(DATOS!$C$57="SÍ",MAX(0.9*$C$23,0.8*$C$22),$C$23)</f>
-        <v>0.1645714285714286</v>
+        <v>0.18514285714285714</v>
       </c>
       <c r="D27" s="19">
         <f>IF(DATOS!$C$57="SÍ",MAX(0.9*$D$23,0.8*$D$22),$D$23)</f>
-        <v>0.17902824552838464</v>
+        <v>0.18514285714285714</v>
       </c>
       <c r="E27" s="6" t="s">
         <v>43</v>
@@ -13106,11 +13106,11 @@
       </c>
       <c r="C28" s="19">
         <f>$C$23*DATOS!$C$12</f>
-        <v>0.23533714285714288</v>
+        <v>0.29417142857142853</v>
       </c>
       <c r="D28" s="19">
         <f>$D$23*DATOS!$C$12</f>
-        <v>0.28445599011732225</v>
+        <v>0.29417142857142853</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>43</v>
@@ -13433,11 +13433,11 @@
       </c>
       <c r="C45" s="13">
         <f>MAX(0.01,IF(DATOS!$C$58&gt;0,MIN(DATOS!$C$58,$C$44*$C$43),$C$43))</f>
-        <v>0.6403056953544697</v>
+        <v>0.334</v>
       </c>
       <c r="D45" s="13">
         <f>MAX(0.01,IF(DATOS!$C$59&gt;0,MIN(DATOS!$C$59,$D$44*$D$43),$D$43))</f>
-        <v>0.631</v>
+        <v>0.125</v>
       </c>
       <c r="E45" s="6" t="s">
         <v>79</v>
@@ -13477,11 +13477,11 @@
       </c>
       <c r="C47" s="19">
         <f>IF($C$45&lt;=DATOS!$C$44,DATOS!$C$41/($C$45*$C$35/DATOS!$C$46),DATOS!$C$41*DATOS!$C$44/($C$45^2*$C$35/DATOS!$C$46))</f>
-        <v>0.5994160704709162</v>
+        <v>1.1491303108069575</v>
       </c>
       <c r="D47" s="19">
         <f>IF($D$45&lt;=DATOS!$C$44,DATOS!$C$41/($D$45*$D$35/DATOS!$C$46),DATOS!$C$41*DATOS!$C$44/($D$45^2*$D$35/DATOS!$C$46))</f>
-        <v>0.6082559806807033</v>
+        <v>3.07047619047619</v>
       </c>
       <c r="E47" s="6" t="s">
         <v>43</v>
@@ -13565,11 +13565,11 @@
       </c>
       <c r="C51" s="21">
         <f>$C$50*DATOS!$C$61</f>
-        <v>8.36466057142857</v>
+        <v>10.577657752380949</v>
       </c>
       <c r="D51" s="21">
         <f>$D$50*DATOS!$C$61</f>
-        <v>8.36466057142857</v>
+        <v>10.577657752380949</v>
       </c>
       <c r="E51" s="6" t="s">
         <v>168</v>
@@ -13587,11 +13587,11 @@
       </c>
       <c r="C52" s="7">
         <f>IF($C$45&lt;=0.5,1,IF($C$45&gt;=2.5,2,1+($C$45-0.5)/2))</f>
-        <v>1.0701528476772348</v>
+        <v>1.0</v>
       </c>
       <c r="D52" s="7">
         <f>IF($D$45&lt;=0.5,1,IF($D$45&gt;=2.5,2,1+($D$45-0.5)/2))</f>
-        <v>1.0655000000000001</v>
+        <v>1.0</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>43</v>
@@ -13716,11 +13716,11 @@
       </c>
       <c r="C60" s="13">
         <f>$C$24*DATOS!$C$12</f>
-        <v>4.031325257142857</v>
+        <v>6.372341485714285</v>
       </c>
       <c r="D60" s="13">
         <f>$D$24*DATOS!$C$12</f>
-        <v>4.872731110709729</v>
+        <v>6.372341485714285</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>168</v>
@@ -13738,11 +13738,11 @@
       </c>
       <c r="C61" s="13">
         <f>$C$51</f>
-        <v>8.36466057142857</v>
+        <v>10.577657752380949</v>
       </c>
       <c r="D61" s="13">
         <f>$D$51</f>
-        <v>8.36466057142857</v>
+        <v>10.577657752380949</v>
       </c>
       <c r="E61" s="6" t="s">
         <v>168</v>
@@ -13760,11 +13760,11 @@
       </c>
       <c r="C62" s="7">
         <f>IF($C$60&gt;0,$C$61/$C$60,0)</f>
-        <v>2.0749158249158244</v>
+        <v>1.6599326599326596</v>
       </c>
       <c r="D62" s="7">
         <f>IF($D$60&gt;0,$D$61/$D$60,0)</f>
-        <v>1.7166267502518169</v>
+        <v>1.6599326599326596</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>43</v>
@@ -13972,10 +13972,10 @@
         </is>
       </c>
       <c r="C73" s="16">
-        <v>1.601</v>
+        <v>2.769</v>
       </c>
       <c r="D73" s="16">
-        <v>2.706</v>
+        <v>2.322</v>
       </c>
       <c r="E73" s="6" t="inlineStr">
         <is>
@@ -14001,11 +14001,11 @@
       </c>
       <c r="C74" s="13">
         <f>$C$27*DATOS!$C$60</f>
-        <v>2.8191085714285715</v>
+        <v>4.010564571428571</v>
       </c>
       <c r="D74" s="13">
         <f>$D$27*DATOS!$C$60</f>
-        <v>3.066753845901229</v>
+        <v>4.010564571428571</v>
       </c>
       <c r="E74" s="6" t="inlineStr">
         <is>
@@ -14061,11 +14061,11 @@
       </c>
       <c r="C76" s="50">
         <f>IF($C$73&gt;0,MAX(1,$C$74/$C$73),1)</f>
-        <v>1.7608423306861785</v>
+        <v>1.4483801269153378</v>
       </c>
       <c r="D76" s="50">
         <f>IF($D$73&gt;0,MAX(1,$D$74/$D$73),1)</f>
-        <v>1.1333162771253618</v>
+        <v>1.7272026578073085</v>
       </c>
       <c r="E76" s="6" t="inlineStr">
         <is>
@@ -14119,11 +14119,11 @@
       </c>
       <c r="C78" s="21">
         <f>$C$76</f>
-        <v>1.7608423306861785</v>
+        <v>1.4483801269153378</v>
       </c>
       <c r="D78" s="21">
         <f>$D$76</f>
-        <v>1.1333162771253618</v>
+        <v>1.7272026578073085</v>
       </c>
       <c r="E78" s="6" t="inlineStr">
         <is>
@@ -14149,11 +14149,11 @@
       </c>
       <c r="C79" s="13">
         <f>IF(DATOS!$C$57="SÍ",0.9,1)*$C$21*DATOS!$C$60</f>
-        <v>2.4402293749461736</v>
+        <v>4.010564571428571</v>
       </c>
       <c r="D79" s="13">
         <f>IF(DATOS!$C$57="SÍ",0.9,1)*$D$21*DATOS!$C$60</f>
-        <v>3.066753845901229</v>
+        <v>4.010564571428571</v>
       </c>
       <c r="E79" s="6" t="inlineStr">
         <is>
@@ -14179,11 +14179,11 @@
       </c>
       <c r="C80" s="21">
         <f>IF($C$73&gt;0,MAX(1,$C$79/$C$73),1)</f>
-        <v>1.524190740128778</v>
+        <v>1.4483801269153378</v>
       </c>
       <c r="D80" s="21">
         <f>IF($D$73&gt;0,MAX(1,$D$79/$D$73),1)</f>
-        <v>1.1333162771253618</v>
+        <v>1.7272026578073085</v>
       </c>
       <c r="E80" s="6" t="inlineStr">
         <is>
@@ -14277,7 +14277,7 @@
       </c>
       <c r="C86" s="13">
         <f>DATOS!$C$60</f>
-        <v>17.13</v>
+        <v>21.662</v>
       </c>
       <c r="D86" s="53">
         <v>17.12906</v>
@@ -14289,7 +14289,7 @@
       </c>
       <c r="F86" s="44" t="inlineStr">
         <is>
-          <t>Tú: CAPTURA de STAAD, DYNAMIC WEIGHT (.anl). Él: E165.</t>
+          <t>Tú: CAPTURA de STAAD, DYNAMIC WEIGHT (.anl R3.0). Él: E165 (modelo sin contravientos).</t>
         </is>
       </c>
       <c r="G86" s="48" t="inlineStr">
@@ -14306,7 +14306,7 @@
       </c>
       <c r="C87" s="13">
         <f>DATOS!$C$58</f>
-        <v>0.889</v>
+        <v>0.334</v>
       </c>
       <c r="D87" s="53">
         <v>0.81</v>
@@ -14335,7 +14335,7 @@
       </c>
       <c r="C88" s="55">
         <f>$C$21</f>
-        <v>0.15828172633756074</v>
+        <v>0.2057142857142857</v>
       </c>
       <c r="D88" s="54">
         <v>0.1684128685092748</v>
@@ -14394,7 +14394,7 @@
       </c>
       <c r="C90" s="55">
         <f>$C$27</f>
-        <v>0.1645714285714286</v>
+        <v>0.18514285714285714</v>
       </c>
       <c r="D90" s="55">
         <f>MAX(0.9*D88,D89)</f>
@@ -14424,7 +14424,7 @@
       </c>
       <c r="C91" s="13">
         <f>$C$74</f>
-        <v>2.8191085714285715</v>
+        <v>4.010564571428571</v>
       </c>
       <c r="D91" s="13">
         <f>D90*D86</f>
@@ -14454,7 +14454,7 @@
       </c>
       <c r="C92" s="13">
         <f>$C$73</f>
-        <v>1.601</v>
+        <v>2.769</v>
       </c>
       <c r="D92" s="53">
         <v>1.82038061</v>
@@ -14483,7 +14483,7 @@
       </c>
       <c r="C93" s="21">
         <f>$C$76</f>
-        <v>1.7608423306861785</v>
+        <v>1.4483801269153378</v>
       </c>
       <c r="D93" s="21">
         <f>MAX(1,D91/D92)</f>
@@ -14525,7 +14525,7 @@
       </c>
       <c r="C95" s="13">
         <f>DATOS!$C$60</f>
-        <v>17.13</v>
+        <v>21.662</v>
       </c>
       <c r="D95" s="53">
         <v>17.12906</v>
@@ -14537,7 +14537,7 @@
       </c>
       <c r="F95" s="44" t="inlineStr">
         <is>
-          <t>Tú: CAPTURA de STAAD, DYNAMIC WEIGHT (.anl). Él: E165.</t>
+          <t>Tú: CAPTURA de STAAD, DYNAMIC WEIGHT (.anl R3.0). Él: E165 (modelo sin contravientos).</t>
         </is>
       </c>
       <c r="G95" s="48" t="inlineStr">
@@ -14554,7 +14554,7 @@
       </c>
       <c r="C96" s="13">
         <f>DATOS!$C$59</f>
-        <v>0.631</v>
+        <v>0.125</v>
       </c>
       <c r="D96" s="53">
         <v>0.63</v>
@@ -14583,7 +14583,7 @@
       </c>
       <c r="C97" s="55">
         <f>$D$21</f>
-        <v>0.19892027280931626</v>
+        <v>0.2057142857142857</v>
       </c>
       <c r="D97" s="54">
         <v>0.1991307148045427</v>
@@ -14642,7 +14642,7 @@
       </c>
       <c r="C99" s="55">
         <f>$D$27</f>
-        <v>0.17902824552838464</v>
+        <v>0.18514285714285714</v>
       </c>
       <c r="D99" s="55">
         <f>MAX(0.9*D97,D98)</f>
@@ -14672,7 +14672,7 @@
       </c>
       <c r="C100" s="13">
         <f>$D$74</f>
-        <v>3.066753845901229</v>
+        <v>4.010564571428571</v>
       </c>
       <c r="D100" s="13">
         <f>D99*D95</f>
@@ -14702,7 +14702,7 @@
       </c>
       <c r="C101" s="13">
         <f>$D$73</f>
-        <v>2.706</v>
+        <v>2.322</v>
       </c>
       <c r="D101" s="53">
         <v>2.72429032</v>
@@ -14731,7 +14731,7 @@
       </c>
       <c r="C102" s="21">
         <f>$D$76</f>
-        <v>1.1333162771253618</v>
+        <v>1.7272026578073085</v>
       </c>
       <c r="D102" s="21">
         <f>MAX(1,D100/D101)</f>
@@ -14793,11 +14793,11 @@
       </c>
       <c r="C104" s="13">
         <f>$C$76</f>
-        <v>1.7608423306861785</v>
+        <v>1.4483801269153378</v>
       </c>
       <c r="D104" s="13">
         <f>$D$76</f>
-        <v>1.1333162771253618</v>
+        <v>1.7272026578073085</v>
       </c>
       <c r="E104" s="6" t="inlineStr">
         <is>
@@ -14823,11 +14823,11 @@
       </c>
       <c r="C105" s="13">
         <f>-$C$76</f>
-        <v>-1.7608423306861785</v>
+        <v>-1.4483801269153378</v>
       </c>
       <c r="D105" s="13">
         <f>-$D$76</f>
-        <v>-1.1333162771253618</v>
+        <v>-1.7272026578073085</v>
       </c>
       <c r="E105" s="6" t="inlineStr">
         <is>
@@ -14853,11 +14853,11 @@
       </c>
       <c r="C106" s="55">
         <f>DATOS!$C$26/$C$12*$C$76</f>
-        <v>0.3622304223125853</v>
+        <v>0.2979524832511552</v>
       </c>
       <c r="D106" s="55">
         <f>DATOS!$C$26/$D$12*$D$76</f>
-        <v>0.23313934843721726</v>
+        <v>0.3553102610346463</v>
       </c>
       <c r="E106" s="6" t="inlineStr">
         <is>
@@ -22184,11 +22184,11 @@
       </c>
       <c r="C9" s="21">
         <f>COEFICIENTE!$C$24</f>
-        <v>2.8191085714285715</v>
+        <v>4.456182857142857</v>
       </c>
       <c r="D9" s="21">
         <f>COEFICIENTE!$D$24</f>
-        <v>3.407504273223587</v>
+        <v>4.456182857142857</v>
       </c>
       <c r="E9" s="6" t="s">
         <v>168</v>
@@ -22207,11 +22207,11 @@
       </c>
       <c r="C10" s="7">
         <f>COEFICIENTE!$C$24*9.80665</f>
-        <v>27.646011072</v>
+        <v>43.700225616</v>
       </c>
       <c r="D10" s="7">
         <f>COEFICIENTE!$D$24*9.80665</f>
-        <v>33.41620178100809</v>
+        <v>43.700225616</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>339</v>
@@ -22230,7 +22230,7 @@
       </c>
       <c r="C11" s="13">
         <f>COEFICIENTE!$C$25*COEFICIENTE!$C$24</f>
-        <v>0.17543312640000003</v>
+        <v>0.0</v>
       </c>
       <c r="D11" s="13">
         <f>COEFICIENTE!$D$25*COEFICIENTE!$D$24</f>
@@ -22253,11 +22253,11 @@
       </c>
       <c r="C12" s="13">
         <f>COEFICIENTE!$C$27*DATOS!$C$60</f>
-        <v>2.8191085714285715</v>
+        <v>4.010564571428571</v>
       </c>
       <c r="D12" s="13">
         <f>COEFICIENTE!$D$27*DATOS!$C$60</f>
-        <v>3.066753845901229</v>
+        <v>4.010564571428571</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>168</v>
@@ -22299,11 +22299,11 @@
       </c>
       <c r="C14" s="13">
         <f>COEFICIENTE!$C$51</f>
-        <v>8.36466057142857</v>
+        <v>10.577657752380949</v>
       </c>
       <c r="D14" s="13">
         <f>COEFICIENTE!$D$51</f>
-        <v>8.36466057142857</v>
+        <v>10.577657752380949</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>168</v>
@@ -22322,11 +22322,11 @@
       </c>
       <c r="C15" s="13">
         <f>COEFICIENTE!$C$54*DATOS!$C$61*IF(DATOS!$C$9="SÍ",COEFICIENTE!$C$64,1)</f>
-        <v>8.36466057142857</v>
+        <v>10.577657752380949</v>
       </c>
       <c r="D15" s="13">
         <f>COEFICIENTE!$D$54*DATOS!$C$61*IF(DATOS!$C$9="SÍ",COEFICIENTE!$D$64,1)</f>
-        <v>8.36466057142857</v>
+        <v>10.577657752380949</v>
       </c>
       <c r="E15" s="6" t="s">
         <v>168</v>
@@ -25006,11 +25006,11 @@
       </c>
       <c r="O15" s="21">
         <f>IF(STAAD!$C$17="ASCE 7-16",STAAD!$C$15,STAAD!$C$12)</f>
-        <v>2.8191085714285715</v>
+        <v>4.010564571428571</v>
       </c>
       <c r="P15" s="21">
         <f>IF(STAAD!$C$17="ASCE 7-16",STAAD!$D$15,STAAD!$D$12)</f>
-        <v>3.066753845901229</v>
+        <v>4.010564571428571</v>
       </c>
       <c r="Q15" s="6" t="s">
         <v>168</v>

</xml_diff>

<commit_message>
R3.1: Excel con W, T y V dinamico del .anl R3.1; espectro X 1.461 / Z 1.641
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DXC88k2xtfXzDpyA8FhCSg
</commit_message>
<xml_diff>
--- a/EspectrosSismo_Naves_ElSalvador_NTDS_ASCE_STAAD_R2.9.xlsx
+++ b/EspectrosSismo_Naves_ElSalvador_NTDS_ASCE_STAAD_R2.9.xlsx
@@ -12399,7 +12399,7 @@
         <v>162</v>
       </c>
       <c r="C58" s="16">
-        <v>0.334</v>
+        <v>0.338</v>
       </c>
       <c r="D58" s="6" t="s">
         <v>79</v>
@@ -12418,7 +12418,7 @@
         <v>165</v>
       </c>
       <c r="C59" s="16">
-        <v>0.125</v>
+        <v>0.126</v>
       </c>
       <c r="D59" s="6" t="s">
         <v>79</v>
@@ -12437,14 +12437,14 @@
         <v>167</v>
       </c>
       <c r="C60" s="15">
-        <v>21.662</v>
+        <v>19.5</v>
       </c>
       <c r="D60" s="6" t="s">
         <v>168</v>
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>CAPTURA de STAAD: DYNAMIC WEIGHT X Y Z = 21,662.18 kg (.anl R3.0).</t>
+          <t>CAPTURA de STAAD: DYNAMIC WEIGHT X Y Z = 19,500.23 kg (.anl R3.1).</t>
         </is>
       </c>
       <c r="F60" s="4" t="s">
@@ -12456,7 +12456,7 @@
         <v>170</v>
       </c>
       <c r="C61" s="15">
-        <v>21.662</v>
+        <v>19.5</v>
       </c>
       <c r="D61" s="6" t="s">
         <v>168</v>
@@ -12908,11 +12908,11 @@
       </c>
       <c r="C19" s="13">
         <f>IF(DATOS!$C$58&gt;0,DATOS!$C$58,$C$18)</f>
-        <v>0.334</v>
+        <v>0.338</v>
       </c>
       <c r="D19" s="13">
         <f>IF(DATOS!$C$59&gt;0,DATOS!$C$59,$D$18)</f>
-        <v>0.125</v>
+        <v>0.126</v>
       </c>
       <c r="E19" s="6" t="s">
         <v>79</v>
@@ -13018,11 +13018,11 @@
       </c>
       <c r="C24" s="21">
         <f>$C$23*DATOS!$C$60</f>
-        <v>4.456182857142857</v>
+        <v>4.011428571428572</v>
       </c>
       <c r="D24" s="21">
         <f>$D$23*DATOS!$C$60</f>
-        <v>4.456182857142857</v>
+        <v>4.011428571428572</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>168</v>
@@ -13433,11 +13433,11 @@
       </c>
       <c r="C45" s="13">
         <f>MAX(0.01,IF(DATOS!$C$58&gt;0,MIN(DATOS!$C$58,$C$44*$C$43),$C$43))</f>
-        <v>0.334</v>
+        <v>0.338</v>
       </c>
       <c r="D45" s="13">
         <f>MAX(0.01,IF(DATOS!$C$59&gt;0,MIN(DATOS!$C$59,$D$44*$D$43),$D$43))</f>
-        <v>0.125</v>
+        <v>0.126</v>
       </c>
       <c r="E45" s="6" t="s">
         <v>79</v>
@@ -13477,11 +13477,11 @@
       </c>
       <c r="C47" s="19">
         <f>IF($C$45&lt;=DATOS!$C$44,DATOS!$C$41/($C$45*$C$35/DATOS!$C$46),DATOS!$C$41*DATOS!$C$44/($C$45^2*$C$35/DATOS!$C$46))</f>
-        <v>1.1491303108069575</v>
+        <v>1.1355311355311355</v>
       </c>
       <c r="D47" s="19">
         <f>IF($D$45&lt;=DATOS!$C$44,DATOS!$C$41/($D$45*$D$35/DATOS!$C$46),DATOS!$C$41*DATOS!$C$44/($D$45^2*$D$35/DATOS!$C$46))</f>
-        <v>3.07047619047619</v>
+        <v>3.0461073318216174</v>
       </c>
       <c r="E47" s="6" t="s">
         <v>43</v>
@@ -13565,11 +13565,11 @@
       </c>
       <c r="C51" s="21">
         <f>$C$50*DATOS!$C$61</f>
-        <v>10.577657752380949</v>
+        <v>9.521942857142855</v>
       </c>
       <c r="D51" s="21">
         <f>$D$50*DATOS!$C$61</f>
-        <v>10.577657752380949</v>
+        <v>9.521942857142855</v>
       </c>
       <c r="E51" s="6" t="s">
         <v>168</v>
@@ -13716,11 +13716,11 @@
       </c>
       <c r="C60" s="13">
         <f>$C$24*DATOS!$C$12</f>
-        <v>6.372341485714285</v>
+        <v>5.736342857142857</v>
       </c>
       <c r="D60" s="13">
         <f>$D$24*DATOS!$C$12</f>
-        <v>6.372341485714285</v>
+        <v>5.736342857142857</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>168</v>
@@ -13738,11 +13738,11 @@
       </c>
       <c r="C61" s="13">
         <f>$C$51</f>
-        <v>10.577657752380949</v>
+        <v>9.521942857142855</v>
       </c>
       <c r="D61" s="13">
         <f>$D$51</f>
-        <v>10.577657752380949</v>
+        <v>9.521942857142855</v>
       </c>
       <c r="E61" s="6" t="s">
         <v>168</v>
@@ -13760,11 +13760,11 @@
       </c>
       <c r="C62" s="7">
         <f>IF($C$60&gt;0,$C$61/$C$60,0)</f>
-        <v>1.6599326599326596</v>
+        <v>1.6599326599326598</v>
       </c>
       <c r="D62" s="7">
         <f>IF($D$60&gt;0,$D$61/$D$60,0)</f>
-        <v>1.6599326599326596</v>
+        <v>1.6599326599326598</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>43</v>
@@ -13972,10 +13972,10 @@
         </is>
       </c>
       <c r="C73" s="16">
-        <v>2.769</v>
+        <v>2.472</v>
       </c>
       <c r="D73" s="16">
-        <v>2.322</v>
+        <v>2.2</v>
       </c>
       <c r="E73" s="6" t="inlineStr">
         <is>
@@ -14001,11 +14001,11 @@
       </c>
       <c r="C74" s="13">
         <f>$C$27*DATOS!$C$60</f>
-        <v>4.010564571428571</v>
+        <v>3.6102857142857143</v>
       </c>
       <c r="D74" s="13">
         <f>$D$27*DATOS!$C$60</f>
-        <v>4.010564571428571</v>
+        <v>3.6102857142857143</v>
       </c>
       <c r="E74" s="6" t="inlineStr">
         <is>
@@ -14061,11 +14061,11 @@
       </c>
       <c r="C76" s="50">
         <f>IF($C$73&gt;0,MAX(1,$C$74/$C$73),1)</f>
-        <v>1.4483801269153378</v>
+        <v>1.4604715672676838</v>
       </c>
       <c r="D76" s="50">
         <f>IF($D$73&gt;0,MAX(1,$D$74/$D$73),1)</f>
-        <v>1.7272026578073085</v>
+        <v>1.6410389610389609</v>
       </c>
       <c r="E76" s="6" t="inlineStr">
         <is>
@@ -14119,11 +14119,11 @@
       </c>
       <c r="C78" s="21">
         <f>$C$76</f>
-        <v>1.4483801269153378</v>
+        <v>1.4604715672676838</v>
       </c>
       <c r="D78" s="21">
         <f>$D$76</f>
-        <v>1.7272026578073085</v>
+        <v>1.6410389610389609</v>
       </c>
       <c r="E78" s="6" t="inlineStr">
         <is>
@@ -14149,11 +14149,11 @@
       </c>
       <c r="C79" s="13">
         <f>IF(DATOS!$C$57="SÍ",0.9,1)*$C$21*DATOS!$C$60</f>
-        <v>4.010564571428571</v>
+        <v>3.6102857142857143</v>
       </c>
       <c r="D79" s="13">
         <f>IF(DATOS!$C$57="SÍ",0.9,1)*$D$21*DATOS!$C$60</f>
-        <v>4.010564571428571</v>
+        <v>3.6102857142857143</v>
       </c>
       <c r="E79" s="6" t="inlineStr">
         <is>
@@ -14179,11 +14179,11 @@
       </c>
       <c r="C80" s="21">
         <f>IF($C$73&gt;0,MAX(1,$C$79/$C$73),1)</f>
-        <v>1.4483801269153378</v>
+        <v>1.4604715672676838</v>
       </c>
       <c r="D80" s="21">
         <f>IF($D$73&gt;0,MAX(1,$D$79/$D$73),1)</f>
-        <v>1.7272026578073085</v>
+        <v>1.6410389610389609</v>
       </c>
       <c r="E80" s="6" t="inlineStr">
         <is>
@@ -14277,7 +14277,7 @@
       </c>
       <c r="C86" s="13">
         <f>DATOS!$C$60</f>
-        <v>21.662</v>
+        <v>19.5</v>
       </c>
       <c r="D86" s="53">
         <v>17.12906</v>
@@ -14289,7 +14289,7 @@
       </c>
       <c r="F86" s="44" t="inlineStr">
         <is>
-          <t>Tú: CAPTURA de STAAD, DYNAMIC WEIGHT (.anl R3.0). Él: E165 (modelo sin contravientos).</t>
+          <t>Tú: CAPTURA de STAAD, DYNAMIC WEIGHT (.anl R3.1). Él: E165 (modelo sin contravientos).</t>
         </is>
       </c>
       <c r="G86" s="48" t="inlineStr">
@@ -14306,7 +14306,7 @@
       </c>
       <c r="C87" s="13">
         <f>DATOS!$C$58</f>
-        <v>0.334</v>
+        <v>0.338</v>
       </c>
       <c r="D87" s="53">
         <v>0.81</v>
@@ -14424,7 +14424,7 @@
       </c>
       <c r="C91" s="13">
         <f>$C$74</f>
-        <v>4.010564571428571</v>
+        <v>3.6102857142857143</v>
       </c>
       <c r="D91" s="13">
         <f>D90*D86</f>
@@ -14454,7 +14454,7 @@
       </c>
       <c r="C92" s="13">
         <f>$C$73</f>
-        <v>2.769</v>
+        <v>2.472</v>
       </c>
       <c r="D92" s="53">
         <v>1.82038061</v>
@@ -14483,7 +14483,7 @@
       </c>
       <c r="C93" s="21">
         <f>$C$76</f>
-        <v>1.4483801269153378</v>
+        <v>1.4604715672676838</v>
       </c>
       <c r="D93" s="21">
         <f>MAX(1,D91/D92)</f>
@@ -14525,7 +14525,7 @@
       </c>
       <c r="C95" s="13">
         <f>DATOS!$C$60</f>
-        <v>21.662</v>
+        <v>19.5</v>
       </c>
       <c r="D95" s="53">
         <v>17.12906</v>
@@ -14537,7 +14537,7 @@
       </c>
       <c r="F95" s="44" t="inlineStr">
         <is>
-          <t>Tú: CAPTURA de STAAD, DYNAMIC WEIGHT (.anl R3.0). Él: E165 (modelo sin contravientos).</t>
+          <t>Tú: CAPTURA de STAAD, DYNAMIC WEIGHT (.anl R3.1). Él: E165 (modelo sin contravientos).</t>
         </is>
       </c>
       <c r="G95" s="48" t="inlineStr">
@@ -14554,7 +14554,7 @@
       </c>
       <c r="C96" s="13">
         <f>DATOS!$C$59</f>
-        <v>0.125</v>
+        <v>0.126</v>
       </c>
       <c r="D96" s="53">
         <v>0.63</v>
@@ -14672,7 +14672,7 @@
       </c>
       <c r="C100" s="13">
         <f>$D$74</f>
-        <v>4.010564571428571</v>
+        <v>3.6102857142857143</v>
       </c>
       <c r="D100" s="13">
         <f>D99*D95</f>
@@ -14702,7 +14702,7 @@
       </c>
       <c r="C101" s="13">
         <f>$D$73</f>
-        <v>2.322</v>
+        <v>2.2</v>
       </c>
       <c r="D101" s="53">
         <v>2.72429032</v>
@@ -14731,7 +14731,7 @@
       </c>
       <c r="C102" s="21">
         <f>$D$76</f>
-        <v>1.7272026578073085</v>
+        <v>1.6410389610389609</v>
       </c>
       <c r="D102" s="21">
         <f>MAX(1,D100/D101)</f>
@@ -14793,11 +14793,11 @@
       </c>
       <c r="C104" s="13">
         <f>$C$76</f>
-        <v>1.4483801269153378</v>
+        <v>1.4604715672676838</v>
       </c>
       <c r="D104" s="13">
         <f>$D$76</f>
-        <v>1.7272026578073085</v>
+        <v>1.6410389610389609</v>
       </c>
       <c r="E104" s="6" t="inlineStr">
         <is>
@@ -14823,11 +14823,11 @@
       </c>
       <c r="C105" s="13">
         <f>-$C$76</f>
-        <v>-1.4483801269153378</v>
+        <v>-1.4604715672676838</v>
       </c>
       <c r="D105" s="13">
         <f>-$D$76</f>
-        <v>-1.7272026578073085</v>
+        <v>-1.6410389610389609</v>
       </c>
       <c r="E105" s="6" t="inlineStr">
         <is>
@@ -14853,11 +14853,11 @@
       </c>
       <c r="C106" s="55">
         <f>DATOS!$C$26/$C$12*$C$76</f>
-        <v>0.2979524832511552</v>
+        <v>0.30043986526649497</v>
       </c>
       <c r="D106" s="55">
         <f>DATOS!$C$26/$D$12*$D$76</f>
-        <v>0.3553102610346463</v>
+        <v>0.33758515769944336</v>
       </c>
       <c r="E106" s="6" t="inlineStr">
         <is>
@@ -22184,11 +22184,11 @@
       </c>
       <c r="C9" s="21">
         <f>COEFICIENTE!$C$24</f>
-        <v>4.456182857142857</v>
+        <v>4.011428571428572</v>
       </c>
       <c r="D9" s="21">
         <f>COEFICIENTE!$D$24</f>
-        <v>4.456182857142857</v>
+        <v>4.011428571428572</v>
       </c>
       <c r="E9" s="6" t="s">
         <v>168</v>
@@ -22207,11 +22207,11 @@
       </c>
       <c r="C10" s="7">
         <f>COEFICIENTE!$C$24*9.80665</f>
-        <v>43.700225616</v>
+        <v>39.338676</v>
       </c>
       <c r="D10" s="7">
         <f>COEFICIENTE!$D$24*9.80665</f>
-        <v>43.700225616</v>
+        <v>39.338676</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>339</v>
@@ -22253,11 +22253,11 @@
       </c>
       <c r="C12" s="13">
         <f>COEFICIENTE!$C$27*DATOS!$C$60</f>
-        <v>4.010564571428571</v>
+        <v>3.6102857142857143</v>
       </c>
       <c r="D12" s="13">
         <f>COEFICIENTE!$D$27*DATOS!$C$60</f>
-        <v>4.010564571428571</v>
+        <v>3.6102857142857143</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>168</v>
@@ -22299,11 +22299,11 @@
       </c>
       <c r="C14" s="13">
         <f>COEFICIENTE!$C$51</f>
-        <v>10.577657752380949</v>
+        <v>9.521942857142855</v>
       </c>
       <c r="D14" s="13">
         <f>COEFICIENTE!$D$51</f>
-        <v>10.577657752380949</v>
+        <v>9.521942857142855</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>168</v>
@@ -22322,11 +22322,11 @@
       </c>
       <c r="C15" s="13">
         <f>COEFICIENTE!$C$54*DATOS!$C$61*IF(DATOS!$C$9="SÍ",COEFICIENTE!$C$64,1)</f>
-        <v>10.577657752380949</v>
+        <v>9.521942857142855</v>
       </c>
       <c r="D15" s="13">
         <f>COEFICIENTE!$D$54*DATOS!$C$61*IF(DATOS!$C$9="SÍ",COEFICIENTE!$D$64,1)</f>
-        <v>10.577657752380949</v>
+        <v>9.521942857142855</v>
       </c>
       <c r="E15" s="6" t="s">
         <v>168</v>
@@ -25006,11 +25006,11 @@
       </c>
       <c r="O15" s="21">
         <f>IF(STAAD!$C$17="ASCE 7-16",STAAD!$C$15,STAAD!$C$12)</f>
-        <v>4.010564571428571</v>
+        <v>3.6102857142857143</v>
       </c>
       <c r="P15" s="21">
         <f>IF(STAAD!$C$17="ASCE 7-16",STAAD!$D$15,STAAD!$D$12)</f>
-        <v>4.010564571428571</v>
+        <v>3.6102857142857143</v>
       </c>
       <c r="Q15" s="6" t="s">
         <v>168</v>

</xml_diff>

<commit_message>
R3.1: Excel y espectro con masa de contravientos en cabezas (X 1.308 / Z 1.593)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DXC88k2xtfXzDpyA8FhCSg
</commit_message>
<xml_diff>
--- a/EspectrosSismo_Naves_ElSalvador_NTDS_ASCE_STAAD_R2.9.xlsx
+++ b/EspectrosSismo_Naves_ElSalvador_NTDS_ASCE_STAAD_R2.9.xlsx
@@ -12399,7 +12399,7 @@
         <v>162</v>
       </c>
       <c r="C58" s="16">
-        <v>0.338</v>
+        <v>0.355</v>
       </c>
       <c r="D58" s="6" t="s">
         <v>79</v>
@@ -12418,7 +12418,7 @@
         <v>165</v>
       </c>
       <c r="C59" s="16">
-        <v>0.126</v>
+        <v>0.128</v>
       </c>
       <c r="D59" s="6" t="s">
         <v>79</v>
@@ -12437,14 +12437,14 @@
         <v>167</v>
       </c>
       <c r="C60" s="15">
-        <v>19.5</v>
+        <v>19.692</v>
       </c>
       <c r="D60" s="6" t="s">
         <v>168</v>
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>CAPTURA de STAAD: DYNAMIC WEIGHT X Y Z = 19,500.23 kg (.anl R3.1).</t>
+          <t>CAPTURA de STAAD: DYNAMIC WEIGHT X Y Z = 19,691.90 kg (.anl R3.1, masa de contravientos en cabezas de columna).</t>
         </is>
       </c>
       <c r="F60" s="4" t="s">
@@ -12456,7 +12456,7 @@
         <v>170</v>
       </c>
       <c r="C61" s="15">
-        <v>19.5</v>
+        <v>19.692</v>
       </c>
       <c r="D61" s="6" t="s">
         <v>168</v>
@@ -12908,11 +12908,11 @@
       </c>
       <c r="C19" s="13">
         <f>IF(DATOS!$C$58&gt;0,DATOS!$C$58,$C$18)</f>
-        <v>0.338</v>
+        <v>0.355</v>
       </c>
       <c r="D19" s="13">
         <f>IF(DATOS!$C$59&gt;0,DATOS!$C$59,$D$18)</f>
-        <v>0.126</v>
+        <v>0.128</v>
       </c>
       <c r="E19" s="6" t="s">
         <v>79</v>
@@ -13018,11 +13018,11 @@
       </c>
       <c r="C24" s="21">
         <f>$C$23*DATOS!$C$60</f>
-        <v>4.011428571428572</v>
+        <v>4.0509257142857145</v>
       </c>
       <c r="D24" s="21">
         <f>$D$23*DATOS!$C$60</f>
-        <v>4.011428571428572</v>
+        <v>4.0509257142857145</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>168</v>
@@ -13433,11 +13433,11 @@
       </c>
       <c r="C45" s="13">
         <f>MAX(0.01,IF(DATOS!$C$58&gt;0,MIN(DATOS!$C$58,$C$44*$C$43),$C$43))</f>
-        <v>0.338</v>
+        <v>0.355</v>
       </c>
       <c r="D45" s="13">
         <f>MAX(0.01,IF(DATOS!$C$59&gt;0,MIN(DATOS!$C$59,$D$44*$D$43),$D$43))</f>
-        <v>0.126</v>
+        <v>0.128</v>
       </c>
       <c r="E45" s="6" t="s">
         <v>79</v>
@@ -13477,11 +13477,11 @@
       </c>
       <c r="C47" s="19">
         <f>IF($C$45&lt;=DATOS!$C$44,DATOS!$C$41/($C$45*$C$35/DATOS!$C$46),DATOS!$C$41*DATOS!$C$44/($C$45^2*$C$35/DATOS!$C$46))</f>
-        <v>1.1355311355311355</v>
+        <v>1.0811535881958416</v>
       </c>
       <c r="D47" s="19">
         <f>IF($D$45&lt;=DATOS!$C$44,DATOS!$C$41/($D$45*$D$35/DATOS!$C$46),DATOS!$C$41*DATOS!$C$44/($D$45^2*$D$35/DATOS!$C$46))</f>
-        <v>3.0461073318216174</v>
+        <v>2.9985119047619047</v>
       </c>
       <c r="E47" s="6" t="s">
         <v>43</v>
@@ -13565,11 +13565,11 @@
       </c>
       <c r="C51" s="21">
         <f>$C$50*DATOS!$C$61</f>
-        <v>9.521942857142855</v>
+        <v>9.615697371428569</v>
       </c>
       <c r="D51" s="21">
         <f>$D$50*DATOS!$C$61</f>
-        <v>9.521942857142855</v>
+        <v>9.615697371428569</v>
       </c>
       <c r="E51" s="6" t="s">
         <v>168</v>
@@ -13716,11 +13716,11 @@
       </c>
       <c r="C60" s="13">
         <f>$C$24*DATOS!$C$12</f>
-        <v>5.736342857142857</v>
+        <v>5.792823771428571</v>
       </c>
       <c r="D60" s="13">
         <f>$D$24*DATOS!$C$12</f>
-        <v>5.736342857142857</v>
+        <v>5.792823771428571</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>168</v>
@@ -13738,11 +13738,11 @@
       </c>
       <c r="C61" s="13">
         <f>$C$51</f>
-        <v>9.521942857142855</v>
+        <v>9.615697371428569</v>
       </c>
       <c r="D61" s="13">
         <f>$D$51</f>
-        <v>9.521942857142855</v>
+        <v>9.615697371428569</v>
       </c>
       <c r="E61" s="6" t="s">
         <v>168</v>
@@ -13760,11 +13760,11 @@
       </c>
       <c r="C62" s="7">
         <f>IF($C$60&gt;0,$C$61/$C$60,0)</f>
-        <v>1.6599326599326598</v>
+        <v>1.6599326599326596</v>
       </c>
       <c r="D62" s="7">
         <f>IF($D$60&gt;0,$D$61/$D$60,0)</f>
-        <v>1.6599326599326598</v>
+        <v>1.6599326599326596</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>43</v>
@@ -13972,10 +13972,10 @@
         </is>
       </c>
       <c r="C73" s="16">
-        <v>2.472</v>
+        <v>2.788</v>
       </c>
       <c r="D73" s="16">
-        <v>2.2</v>
+        <v>2.29</v>
       </c>
       <c r="E73" s="6" t="inlineStr">
         <is>
@@ -14001,11 +14001,11 @@
       </c>
       <c r="C74" s="13">
         <f>$C$27*DATOS!$C$60</f>
-        <v>3.6102857142857143</v>
+        <v>3.6458331428571427</v>
       </c>
       <c r="D74" s="13">
         <f>$D$27*DATOS!$C$60</f>
-        <v>3.6102857142857143</v>
+        <v>3.6458331428571427</v>
       </c>
       <c r="E74" s="6" t="inlineStr">
         <is>
@@ -14061,11 +14061,11 @@
       </c>
       <c r="C76" s="50">
         <f>IF($C$73&gt;0,MAX(1,$C$74/$C$73),1)</f>
-        <v>1.4604715672676838</v>
+        <v>1.3076876409100227</v>
       </c>
       <c r="D76" s="50">
         <f>IF($D$73&gt;0,MAX(1,$D$74/$D$73),1)</f>
-        <v>1.6410389610389609</v>
+        <v>1.5920668746101059</v>
       </c>
       <c r="E76" s="6" t="inlineStr">
         <is>
@@ -14119,11 +14119,11 @@
       </c>
       <c r="C78" s="21">
         <f>$C$76</f>
-        <v>1.4604715672676838</v>
+        <v>1.3076876409100227</v>
       </c>
       <c r="D78" s="21">
         <f>$D$76</f>
-        <v>1.6410389610389609</v>
+        <v>1.5920668746101059</v>
       </c>
       <c r="E78" s="6" t="inlineStr">
         <is>
@@ -14149,11 +14149,11 @@
       </c>
       <c r="C79" s="13">
         <f>IF(DATOS!$C$57="SÍ",0.9,1)*$C$21*DATOS!$C$60</f>
-        <v>3.6102857142857143</v>
+        <v>3.6458331428571427</v>
       </c>
       <c r="D79" s="13">
         <f>IF(DATOS!$C$57="SÍ",0.9,1)*$D$21*DATOS!$C$60</f>
-        <v>3.6102857142857143</v>
+        <v>3.6458331428571427</v>
       </c>
       <c r="E79" s="6" t="inlineStr">
         <is>
@@ -14179,11 +14179,11 @@
       </c>
       <c r="C80" s="21">
         <f>IF($C$73&gt;0,MAX(1,$C$79/$C$73),1)</f>
-        <v>1.4604715672676838</v>
+        <v>1.3076876409100227</v>
       </c>
       <c r="D80" s="21">
         <f>IF($D$73&gt;0,MAX(1,$D$79/$D$73),1)</f>
-        <v>1.6410389610389609</v>
+        <v>1.5920668746101059</v>
       </c>
       <c r="E80" s="6" t="inlineStr">
         <is>
@@ -14277,7 +14277,7 @@
       </c>
       <c r="C86" s="13">
         <f>DATOS!$C$60</f>
-        <v>19.5</v>
+        <v>19.692</v>
       </c>
       <c r="D86" s="53">
         <v>17.12906</v>
@@ -14306,7 +14306,7 @@
       </c>
       <c r="C87" s="13">
         <f>DATOS!$C$58</f>
-        <v>0.338</v>
+        <v>0.355</v>
       </c>
       <c r="D87" s="53">
         <v>0.81</v>
@@ -14424,7 +14424,7 @@
       </c>
       <c r="C91" s="13">
         <f>$C$74</f>
-        <v>3.6102857142857143</v>
+        <v>3.6458331428571427</v>
       </c>
       <c r="D91" s="13">
         <f>D90*D86</f>
@@ -14454,7 +14454,7 @@
       </c>
       <c r="C92" s="13">
         <f>$C$73</f>
-        <v>2.472</v>
+        <v>2.788</v>
       </c>
       <c r="D92" s="53">
         <v>1.82038061</v>
@@ -14483,7 +14483,7 @@
       </c>
       <c r="C93" s="21">
         <f>$C$76</f>
-        <v>1.4604715672676838</v>
+        <v>1.3076876409100227</v>
       </c>
       <c r="D93" s="21">
         <f>MAX(1,D91/D92)</f>
@@ -14525,7 +14525,7 @@
       </c>
       <c r="C95" s="13">
         <f>DATOS!$C$60</f>
-        <v>19.5</v>
+        <v>19.692</v>
       </c>
       <c r="D95" s="53">
         <v>17.12906</v>
@@ -14554,7 +14554,7 @@
       </c>
       <c r="C96" s="13">
         <f>DATOS!$C$59</f>
-        <v>0.126</v>
+        <v>0.128</v>
       </c>
       <c r="D96" s="53">
         <v>0.63</v>
@@ -14672,7 +14672,7 @@
       </c>
       <c r="C100" s="13">
         <f>$D$74</f>
-        <v>3.6102857142857143</v>
+        <v>3.6458331428571427</v>
       </c>
       <c r="D100" s="13">
         <f>D99*D95</f>
@@ -14702,7 +14702,7 @@
       </c>
       <c r="C101" s="13">
         <f>$D$73</f>
-        <v>2.2</v>
+        <v>2.29</v>
       </c>
       <c r="D101" s="53">
         <v>2.72429032</v>
@@ -14731,7 +14731,7 @@
       </c>
       <c r="C102" s="21">
         <f>$D$76</f>
-        <v>1.6410389610389609</v>
+        <v>1.5920668746101059</v>
       </c>
       <c r="D102" s="21">
         <f>MAX(1,D100/D101)</f>
@@ -14793,11 +14793,11 @@
       </c>
       <c r="C104" s="13">
         <f>$C$76</f>
-        <v>1.4604715672676838</v>
+        <v>1.3076876409100227</v>
       </c>
       <c r="D104" s="13">
         <f>$D$76</f>
-        <v>1.6410389610389609</v>
+        <v>1.5920668746101059</v>
       </c>
       <c r="E104" s="6" t="inlineStr">
         <is>
@@ -14823,11 +14823,11 @@
       </c>
       <c r="C105" s="13">
         <f>-$C$76</f>
-        <v>-1.4604715672676838</v>
+        <v>-1.3076876409100227</v>
       </c>
       <c r="D105" s="13">
         <f>-$D$76</f>
-        <v>-1.6410389610389609</v>
+        <v>-1.5920668746101059</v>
       </c>
       <c r="E105" s="6" t="inlineStr">
         <is>
@@ -14853,11 +14853,11 @@
       </c>
       <c r="C106" s="55">
         <f>DATOS!$C$26/$C$12*$C$76</f>
-        <v>0.30043986526649497</v>
+        <v>0.26901002898720466</v>
       </c>
       <c r="D106" s="55">
         <f>DATOS!$C$26/$D$12*$D$76</f>
-        <v>0.33758515769944336</v>
+        <v>0.3275108999197932</v>
       </c>
       <c r="E106" s="6" t="inlineStr">
         <is>
@@ -22184,11 +22184,11 @@
       </c>
       <c r="C9" s="21">
         <f>COEFICIENTE!$C$24</f>
-        <v>4.011428571428572</v>
+        <v>4.0509257142857145</v>
       </c>
       <c r="D9" s="21">
         <f>COEFICIENTE!$D$24</f>
-        <v>4.011428571428572</v>
+        <v>4.0509257142857145</v>
       </c>
       <c r="E9" s="6" t="s">
         <v>168</v>
@@ -22207,11 +22207,11 @@
       </c>
       <c r="C10" s="7">
         <f>COEFICIENTE!$C$24*9.80665</f>
-        <v>39.338676</v>
+        <v>39.726010656</v>
       </c>
       <c r="D10" s="7">
         <f>COEFICIENTE!$D$24*9.80665</f>
-        <v>39.338676</v>
+        <v>39.726010656</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>339</v>
@@ -22253,11 +22253,11 @@
       </c>
       <c r="C12" s="13">
         <f>COEFICIENTE!$C$27*DATOS!$C$60</f>
-        <v>3.6102857142857143</v>
+        <v>3.6458331428571427</v>
       </c>
       <c r="D12" s="13">
         <f>COEFICIENTE!$D$27*DATOS!$C$60</f>
-        <v>3.6102857142857143</v>
+        <v>3.6458331428571427</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>168</v>
@@ -22299,11 +22299,11 @@
       </c>
       <c r="C14" s="13">
         <f>COEFICIENTE!$C$51</f>
-        <v>9.521942857142855</v>
+        <v>9.615697371428569</v>
       </c>
       <c r="D14" s="13">
         <f>COEFICIENTE!$D$51</f>
-        <v>9.521942857142855</v>
+        <v>9.615697371428569</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>168</v>
@@ -22322,11 +22322,11 @@
       </c>
       <c r="C15" s="13">
         <f>COEFICIENTE!$C$54*DATOS!$C$61*IF(DATOS!$C$9="SÍ",COEFICIENTE!$C$64,1)</f>
-        <v>9.521942857142855</v>
+        <v>9.615697371428569</v>
       </c>
       <c r="D15" s="13">
         <f>COEFICIENTE!$D$54*DATOS!$C$61*IF(DATOS!$C$9="SÍ",COEFICIENTE!$D$64,1)</f>
-        <v>9.521942857142855</v>
+        <v>9.615697371428569</v>
       </c>
       <c r="E15" s="6" t="s">
         <v>168</v>
@@ -25006,11 +25006,11 @@
       </c>
       <c r="O15" s="21">
         <f>IF(STAAD!$C$17="ASCE 7-16",STAAD!$C$15,STAAD!$C$12)</f>
-        <v>3.6102857142857143</v>
+        <v>3.6458331428571427</v>
       </c>
       <c r="P15" s="21">
         <f>IF(STAAD!$C$17="ASCE 7-16",STAAD!$D$15,STAAD!$D$12)</f>
-        <v>3.6102857142857143</v>
+        <v>3.6458331428571427</v>
       </c>
       <c r="Q15" s="6" t="s">
         <v>168</v>

</xml_diff>